<commit_message>
thêm chức năng import
</commit_message>
<xml_diff>
--- a/server/CRM/CRM/wwwroot/Templates/ThongTinTiemNang.xlsx
+++ b/server/CRM/CRM/wwwroot/Templates/ThongTinTiemNang.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MSIs\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CRM\CRM\server\CRM\CRM\wwwroot\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A11899AB-19D2-465A-B487-E43D292A1A53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1D27CCA-E254-4F40-82CC-95DB2AA81A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3108" yWindow="1536" windowWidth="21120" windowHeight="10512" xr2:uid="{97B07EE4-0850-4CD7-A078-E42B6BC90780}"/>
+    <workbookView xWindow="1752" yWindow="576" windowWidth="21120" windowHeight="10512" xr2:uid="{97B07EE4-0850-4CD7-A078-E42B6BC90780}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -85,6 +85,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="m/d/yy\ h:mm;@"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -127,10 +130,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -445,7 +449,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B87B1377-5947-465F-93BB-487646B99284}">
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.88671875" style="2" customWidth="1"/>
@@ -525,6 +529,9 @@
         <v>17</v>
       </c>
     </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="P2" s="3"/>
+    </row>
   </sheetData>
   <dataValidations count="7">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B100" xr:uid="{FD2B4EA1-D9D4-4402-85EF-3B355AF48B83}">

</xml_diff>